<commit_message>
Made some small changes
Made some small changes
</commit_message>
<xml_diff>
--- a/docs/rocket_weight.xlsx
+++ b/docs/rocket_weight.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mainport365-my.sharepoint.com/personal/bzelissen_mainport_nl/Documents/Documenten/Arduino/sketches/ESP-Controlled-Rocket/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="251" documentId="11_F25DC773A252ABDACC10484BC95F46505ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9C8620F-8ED5-4F9F-A88D-52BF68211D89}"/>
+  <xr:revisionPtr revIDLastSave="260" documentId="11_F25DC773A252ABDACC10484BC95F46505ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46635730-9343-49D5-9847-1AE274A1E68C}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="-15960" yWindow="-15480" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-15960" yWindow="-15480" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -682,7 +682,7 @@
         <v>1</v>
       </c>
       <c r="D3" s="9">
-        <f t="shared" ref="D3:J26" si="0">B3*C3</f>
+        <f t="shared" ref="D3:D26" si="0">B3*C3</f>
         <v>23</v>
       </c>
       <c r="E3" s="9">
@@ -1216,14 +1216,14 @@
         <v>32</v>
       </c>
       <c r="B18" s="2">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="C18" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" s="9">
         <f t="shared" ref="D18" si="6">B18*C18</f>
-        <v>114</v>
+        <v>42</v>
       </c>
       <c r="E18" s="9">
         <v>0</v>
@@ -1541,7 +1541,7 @@
       <c r="C27" s="7"/>
       <c r="D27" s="12">
         <f>SUM(D2:D26)</f>
-        <v>302.25</v>
+        <v>230.25</v>
       </c>
       <c r="E27" s="12"/>
       <c r="F27" s="12">
@@ -1560,6 +1560,66 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="B2:B26">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:D26">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F26">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:H26">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J2:J26">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: move dashboard & visualization to SPIFFS + add dual file manager (SD & SPIFFS)
feat: move dashboard & visualization to SPIFFS + add dual file manager (SD & SPIFFS)
</commit_message>
<xml_diff>
--- a/docs/rocket_weight.xlsx
+++ b/docs/rocket_weight.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mainport365-my.sharepoint.com/personal/bzelissen_mainport_nl/Documents/Documenten/Arduino/sketches/ESP-Controlled-Rocket/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="260" documentId="11_F25DC773A252ABDACC10484BC95F46505ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46635730-9343-49D5-9847-1AE274A1E68C}"/>
+  <xr:revisionPtr revIDLastSave="275" documentId="11_F25DC773A252ABDACC10484BC95F46505ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B6EBC718-96DC-4318-A698-E57485299ABC}"/>
   <bookViews>
-    <workbookView xWindow="-15960" yWindow="-15480" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>Part</t>
   </si>
@@ -141,6 +141,12 @@
   </si>
   <si>
     <t>Battery Mount</t>
+  </si>
+  <si>
+    <t># Parts 13.5L Rocket</t>
+  </si>
+  <si>
+    <t>Total weight 13.5L Rocket</t>
   </si>
 </sst>
 </file>
@@ -595,15 +601,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="10" width="13.7109375" style="9" customWidth="1"/>
+    <col min="11" max="11" width="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" s="1" customFormat="1" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -634,8 +641,14 @@
       <c r="J1" s="8" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K1" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -670,8 +683,15 @@
         <f>B2*I2</f>
         <v>19</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K2" s="9">
+        <v>1</v>
+      </c>
+      <c r="L2" s="10">
+        <f t="shared" ref="L2:L26" si="0">B2*K2</f>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -682,68 +702,82 @@
         <v>1</v>
       </c>
       <c r="D3" s="9">
-        <f t="shared" ref="D3:D26" si="0">B3*C3</f>
+        <f t="shared" ref="D3:D26" si="1">B3*C3</f>
         <v>23</v>
       </c>
       <c r="E3" s="9">
         <v>1</v>
       </c>
       <c r="F3" s="9">
-        <f t="shared" ref="F3:F26" si="1">B3*E3</f>
+        <f t="shared" ref="F3:F26" si="2">B3*E3</f>
         <v>23</v>
       </c>
       <c r="G3" s="9">
         <v>1</v>
       </c>
       <c r="H3" s="9">
-        <f t="shared" ref="H3:H26" si="2">B3*G3</f>
+        <f t="shared" ref="H3:H26" si="3">B3*G3</f>
         <v>23</v>
       </c>
       <c r="I3" s="9">
         <v>1</v>
       </c>
       <c r="J3" s="10">
-        <f t="shared" ref="J3:J26" si="3">B3*I3</f>
+        <f t="shared" ref="J3:J26" si="4">B3*I3</f>
         <v>23</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K3" s="9">
+        <v>1</v>
+      </c>
+      <c r="L3" s="10">
+        <f t="shared" si="0"/>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B4" s="2">
-        <v>30.4</v>
+        <v>26</v>
       </c>
       <c r="C4" s="9">
         <v>0</v>
       </c>
       <c r="D4" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E4" s="9">
         <v>1</v>
       </c>
       <c r="F4" s="9">
-        <f t="shared" si="1"/>
-        <v>30.4</v>
+        <f t="shared" si="2"/>
+        <v>26</v>
       </c>
       <c r="G4" s="9">
         <v>2</v>
       </c>
       <c r="H4" s="9">
-        <f t="shared" si="2"/>
-        <v>60.8</v>
+        <f t="shared" si="3"/>
+        <v>52</v>
       </c>
       <c r="I4" s="9">
         <v>3</v>
       </c>
       <c r="J4" s="10">
-        <f t="shared" si="3"/>
-        <v>91.199999999999989</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v>78</v>
+      </c>
+      <c r="K4" s="9">
+        <v>4</v>
+      </c>
+      <c r="L4" s="10">
+        <f t="shared" si="0"/>
+        <v>104</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
@@ -754,68 +788,82 @@
         <v>1</v>
       </c>
       <c r="D5" s="9">
-        <f t="shared" si="0"/>
-        <v>41.25</v>
-      </c>
-      <c r="E5" s="9">
-        <v>1</v>
-      </c>
-      <c r="F5" s="9">
         <f t="shared" si="1"/>
         <v>41.25</v>
       </c>
+      <c r="E5" s="9">
+        <v>1</v>
+      </c>
+      <c r="F5" s="9">
+        <f t="shared" si="2"/>
+        <v>41.25</v>
+      </c>
       <c r="G5" s="9">
         <v>1</v>
       </c>
       <c r="H5" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>41.25</v>
       </c>
       <c r="I5" s="9">
         <v>1</v>
       </c>
       <c r="J5" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>41.25</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K5" s="9">
+        <v>1</v>
+      </c>
+      <c r="L5" s="10">
+        <f t="shared" si="0"/>
+        <v>41.25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B6" s="2">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C6" s="9">
         <v>0</v>
       </c>
       <c r="D6" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E6" s="9">
         <v>1</v>
       </c>
       <c r="F6" s="9">
-        <f t="shared" si="1"/>
-        <v>82</v>
+        <f t="shared" si="2"/>
+        <v>80</v>
       </c>
       <c r="G6" s="9">
         <v>2</v>
       </c>
       <c r="H6" s="9">
-        <f t="shared" si="2"/>
-        <v>164</v>
+        <f t="shared" si="3"/>
+        <v>160</v>
       </c>
       <c r="I6" s="9">
         <v>3</v>
       </c>
       <c r="J6" s="10">
-        <f t="shared" si="3"/>
-        <v>246</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v>240</v>
+      </c>
+      <c r="K6" s="9">
+        <v>4</v>
+      </c>
+      <c r="L6" s="10">
+        <f>B6*K6</f>
+        <v>320</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>29</v>
       </c>
@@ -826,32 +874,39 @@
         <v>1</v>
       </c>
       <c r="D7" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>43</v>
       </c>
       <c r="E7" s="9">
         <v>0</v>
       </c>
       <c r="F7" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="G7" s="9">
         <v>0</v>
       </c>
       <c r="H7" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="I7" s="9">
         <v>0</v>
       </c>
       <c r="J7" s="10">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="K7" s="9">
+        <v>0</v>
+      </c>
+      <c r="L7" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>30</v>
       </c>
@@ -862,32 +917,39 @@
         <v>0</v>
       </c>
       <c r="D8" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E8" s="9">
         <v>1</v>
       </c>
       <c r="F8" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>47</v>
       </c>
       <c r="G8" s="9">
         <v>1</v>
       </c>
       <c r="H8" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>47</v>
       </c>
       <c r="I8" s="9">
         <v>1</v>
       </c>
       <c r="J8" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>47</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K8" s="9">
+        <v>1</v>
+      </c>
+      <c r="L8" s="10">
+        <f t="shared" si="0"/>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>14</v>
       </c>
@@ -905,25 +967,32 @@
         <v>1</v>
       </c>
       <c r="F9" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>74</v>
       </c>
       <c r="G9" s="9">
         <v>1</v>
       </c>
       <c r="H9" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>74</v>
       </c>
       <c r="I9" s="9">
         <v>1</v>
       </c>
       <c r="J9" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>74</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K9" s="9">
+        <v>1</v>
+      </c>
+      <c r="L9" s="10">
+        <f t="shared" si="0"/>
+        <v>74</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>15</v>
       </c>
@@ -934,32 +1003,39 @@
         <v>0</v>
       </c>
       <c r="D10" s="9">
-        <f t="shared" ref="D10:D17" si="4">B10*C10</f>
+        <f t="shared" ref="D10:D17" si="5">B10*C10</f>
         <v>0</v>
       </c>
       <c r="E10" s="9">
         <v>1</v>
       </c>
       <c r="F10" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>40</v>
       </c>
       <c r="G10" s="9">
         <v>1</v>
       </c>
       <c r="H10" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>40</v>
       </c>
       <c r="I10" s="9">
         <v>1</v>
       </c>
       <c r="J10" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>40</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K10" s="9">
+        <v>1</v>
+      </c>
+      <c r="L10" s="10">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>33</v>
       </c>
@@ -970,32 +1046,39 @@
         <v>0</v>
       </c>
       <c r="D11" s="9">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="E11" s="9">
         <v>1</v>
       </c>
       <c r="F11" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>7</v>
       </c>
       <c r="G11" s="9">
         <v>1</v>
       </c>
       <c r="H11" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>7</v>
       </c>
       <c r="I11" s="9">
         <v>1</v>
       </c>
       <c r="J11" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>7</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K11" s="9">
+        <v>1</v>
+      </c>
+      <c r="L11" s="10">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>16</v>
       </c>
@@ -1006,32 +1089,39 @@
         <v>0</v>
       </c>
       <c r="D12" s="9">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="E12" s="9">
         <v>1</v>
       </c>
       <c r="F12" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>97</v>
       </c>
       <c r="G12" s="9">
         <v>1</v>
       </c>
       <c r="H12" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>97</v>
       </c>
       <c r="I12" s="9">
         <v>1</v>
       </c>
       <c r="J12" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>97</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K12" s="9">
+        <v>1</v>
+      </c>
+      <c r="L12" s="10">
+        <f t="shared" si="0"/>
+        <v>97</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>34</v>
       </c>
@@ -1042,32 +1132,39 @@
         <v>0</v>
       </c>
       <c r="D13" s="9">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="E13" s="9">
         <v>1</v>
       </c>
       <c r="F13" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>8</v>
       </c>
       <c r="G13" s="9">
         <v>1</v>
       </c>
       <c r="H13" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>8</v>
       </c>
       <c r="I13" s="9">
         <v>1</v>
       </c>
       <c r="J13" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K13" s="9">
+        <v>1</v>
+      </c>
+      <c r="L13" s="10">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>17</v>
       </c>
@@ -1078,32 +1175,39 @@
         <v>1</v>
       </c>
       <c r="D14" s="9">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>26</v>
       </c>
       <c r="E14" s="9">
         <v>0</v>
       </c>
       <c r="F14" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="G14" s="9">
         <v>0</v>
       </c>
       <c r="H14" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="I14" s="9">
         <v>0</v>
       </c>
       <c r="J14" s="10">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="K14" s="9">
+        <v>0</v>
+      </c>
+      <c r="L14" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>18</v>
       </c>
@@ -1114,32 +1218,39 @@
         <v>0</v>
       </c>
       <c r="D15" s="9">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="E15" s="9">
         <v>0</v>
       </c>
       <c r="F15" s="9">
-        <f t="shared" ref="F15" si="5">B15*E15</f>
+        <f t="shared" ref="F15" si="6">B15*E15</f>
         <v>0</v>
       </c>
       <c r="G15" s="9">
         <v>0</v>
       </c>
       <c r="H15" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="I15" s="9">
         <v>0</v>
       </c>
       <c r="J15" s="10">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="K15" s="9">
+        <v>0</v>
+      </c>
+      <c r="L15" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>19</v>
       </c>
@@ -1150,32 +1261,39 @@
         <v>0</v>
       </c>
       <c r="D16" s="9">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="E16" s="9">
         <v>0</v>
       </c>
       <c r="F16" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="G16" s="9">
         <v>0</v>
       </c>
       <c r="H16" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="I16" s="9">
         <v>0</v>
       </c>
       <c r="J16" s="10">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="K16" s="9">
+        <v>0</v>
+      </c>
+      <c r="L16" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>20</v>
       </c>
@@ -1186,32 +1304,39 @@
         <v>1</v>
       </c>
       <c r="D17" s="9">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>36</v>
       </c>
       <c r="E17" s="9">
         <v>0</v>
       </c>
       <c r="F17" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="G17" s="9">
         <v>0</v>
       </c>
       <c r="H17" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="I17" s="9">
         <v>0</v>
       </c>
       <c r="J17" s="10">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="K17" s="9">
+        <v>0</v>
+      </c>
+      <c r="L17" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>32</v>
       </c>
@@ -1222,140 +1347,168 @@
         <v>1</v>
       </c>
       <c r="D18" s="9">
-        <f t="shared" ref="D18" si="6">B18*C18</f>
+        <f t="shared" ref="D18" si="7">B18*C18</f>
         <v>42</v>
       </c>
       <c r="E18" s="9">
         <v>0</v>
       </c>
       <c r="F18" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="G18" s="9">
         <v>0</v>
       </c>
       <c r="H18" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="I18" s="9">
         <v>0</v>
       </c>
       <c r="J18" s="10">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="K18" s="9">
+        <v>0</v>
+      </c>
+      <c r="L18" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>22</v>
       </c>
       <c r="B19" s="2">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="C19" s="9">
         <v>0</v>
       </c>
       <c r="D19" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E19" s="9">
         <v>1</v>
       </c>
       <c r="F19" s="9">
-        <f t="shared" si="1"/>
-        <v>33</v>
+        <f t="shared" si="2"/>
+        <v>26</v>
       </c>
       <c r="G19" s="9">
         <v>1</v>
       </c>
       <c r="H19" s="9">
-        <f t="shared" si="2"/>
-        <v>33</v>
+        <f t="shared" si="3"/>
+        <v>26</v>
       </c>
       <c r="I19" s="9">
         <v>1</v>
       </c>
       <c r="J19" s="10">
-        <f t="shared" si="3"/>
-        <v>33</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v>26</v>
+      </c>
+      <c r="K19" s="9">
+        <v>1</v>
+      </c>
+      <c r="L19" s="10">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>21</v>
       </c>
       <c r="B20" s="2">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="C20" s="9">
         <v>0</v>
       </c>
       <c r="D20" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E20" s="9">
         <v>1</v>
       </c>
       <c r="F20" s="9">
-        <f t="shared" si="1"/>
-        <v>111</v>
+        <f t="shared" si="2"/>
+        <v>100</v>
       </c>
       <c r="G20" s="9">
         <v>1</v>
       </c>
       <c r="H20" s="9">
-        <f t="shared" si="2"/>
-        <v>111</v>
+        <f t="shared" si="3"/>
+        <v>100</v>
       </c>
       <c r="I20" s="9">
         <v>1</v>
       </c>
       <c r="J20" s="10">
-        <f t="shared" si="3"/>
-        <v>111</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v>100</v>
+      </c>
+      <c r="K20" s="9">
+        <v>1</v>
+      </c>
+      <c r="L20" s="10">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>23</v>
       </c>
       <c r="B21" s="2">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="C21" s="9">
         <v>0</v>
       </c>
       <c r="D21" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E21" s="9">
         <v>1</v>
       </c>
       <c r="F21" s="9">
-        <f t="shared" si="1"/>
-        <v>69</v>
+        <f t="shared" si="2"/>
+        <v>123</v>
       </c>
       <c r="G21" s="9">
         <v>1</v>
       </c>
       <c r="H21" s="9">
-        <f t="shared" si="2"/>
-        <v>69</v>
+        <f t="shared" si="3"/>
+        <v>123</v>
       </c>
       <c r="I21" s="9">
         <v>1</v>
       </c>
       <c r="J21" s="10">
-        <f t="shared" si="3"/>
-        <v>69</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v>123</v>
+      </c>
+      <c r="K21" s="9">
+        <v>1</v>
+      </c>
+      <c r="L21" s="10">
+        <f t="shared" si="0"/>
+        <v>123</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>24</v>
       </c>
@@ -1366,32 +1519,39 @@
         <v>0</v>
       </c>
       <c r="D22" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E22" s="9">
         <v>3</v>
       </c>
       <c r="F22" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>45</v>
       </c>
       <c r="G22" s="9">
         <v>3</v>
       </c>
       <c r="H22" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>45</v>
       </c>
       <c r="I22" s="9">
         <v>3</v>
       </c>
       <c r="J22" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>45</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K22" s="9">
+        <v>3</v>
+      </c>
+      <c r="L22" s="10">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>25</v>
       </c>
@@ -1402,32 +1562,39 @@
         <v>0</v>
       </c>
       <c r="D23" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E23" s="9">
         <v>2</v>
       </c>
       <c r="F23" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
       <c r="G23" s="9">
         <v>2</v>
       </c>
       <c r="H23" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>10</v>
       </c>
       <c r="I23" s="9">
         <v>2</v>
       </c>
       <c r="J23" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>10</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K23" s="9">
+        <v>2</v>
+      </c>
+      <c r="L23" s="10">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>26</v>
       </c>
@@ -1438,32 +1605,39 @@
         <v>0</v>
       </c>
       <c r="D24" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E24" s="9">
         <v>0</v>
       </c>
       <c r="F24" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="G24" s="9">
         <v>0</v>
       </c>
       <c r="H24" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="I24" s="9">
         <v>0</v>
       </c>
       <c r="J24" s="10">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="K24" s="9">
+        <v>0</v>
+      </c>
+      <c r="L24" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>27</v>
       </c>
@@ -1474,32 +1648,39 @@
         <v>0</v>
       </c>
       <c r="D25" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E25" s="9">
         <v>0</v>
       </c>
       <c r="F25" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="G25" s="9">
         <v>0</v>
       </c>
       <c r="H25" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="I25" s="9">
         <v>0</v>
       </c>
       <c r="J25" s="10">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="K25" s="9">
+        <v>0</v>
+      </c>
+      <c r="L25" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
         <v>28</v>
       </c>
@@ -1510,32 +1691,39 @@
         <v>0</v>
       </c>
       <c r="D26" s="11">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E26" s="11">
         <v>1</v>
       </c>
       <c r="F26" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>25</v>
       </c>
       <c r="G26" s="11">
         <v>1</v>
       </c>
       <c r="H26" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>25</v>
       </c>
       <c r="I26" s="11">
         <v>1</v>
       </c>
       <c r="J26" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>25</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="K26" s="11">
+        <v>1</v>
+      </c>
+      <c r="L26" s="10">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="5"/>
       <c r="B27" s="6"/>
       <c r="C27" s="7"/>
@@ -1546,21 +1734,38 @@
       <c r="E27" s="12"/>
       <c r="F27" s="12">
         <f>SUM(F2:F26)</f>
-        <v>761.65</v>
+        <v>791.25</v>
       </c>
       <c r="G27" s="12"/>
       <c r="H27" s="12">
         <f>SUM(H2:H26)</f>
-        <v>874.05</v>
+        <v>897.25</v>
       </c>
       <c r="I27" s="12"/>
       <c r="J27" s="13">
         <f>SUM(J2:J26)</f>
-        <v>986.45</v>
+        <v>1003.25</v>
+      </c>
+      <c r="K27" s="12"/>
+      <c r="L27" s="13">
+        <f>SUM(L2:L26)</f>
+        <v>1109.25</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2:B26">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:D26">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -1572,7 +1777,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D26">
+  <conditionalFormatting sqref="F2:F26">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -1584,7 +1789,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F26">
+  <conditionalFormatting sqref="H2:H26">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -1596,7 +1801,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H26">
+  <conditionalFormatting sqref="J2:J26">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -1608,7 +1813,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J26">
+  <conditionalFormatting sqref="L2:L26">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>